<commit_message>
v9.4 — PADRAO §3.8 (% Vendido) formalizado + validação automática (corrigiu Zion e Vernazza N
</commit_message>
<xml_diff>
--- a/Planilha_Mestre_Panorama_v9.3.xlsx
+++ b/Planilha_Mestre_Panorama_v9.3.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composição" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empreendimentos'!$A$5:$Y$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empreendimentos'!$A$5:$Z$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incorporadoras'!$A$5:$O$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composição'!$A$5:$J$35</definedName>
   </definedNames>
@@ -738,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y53"/>
+  <dimension ref="A1:Z53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -760,12 +760,13 @@
     <col width="11" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="28" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="50" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="28" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="50" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -794,6 +795,7 @@
       <c r="W1" s="1" t="n"/>
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="1" t="n"/>
@@ -913,30 +915,35 @@
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
+          <t>Origem % Vendido</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
           <t>Orig. preços</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="V5" s="4" t="inlineStr">
         <is>
           <t>Orig. estoque</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
+      <c r="W5" s="4" t="inlineStr">
         <is>
           <t>Orig. lançamento</t>
         </is>
       </c>
-      <c r="W5" s="4" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr">
         <is>
           <t>Link fonte principal</t>
         </is>
       </c>
-      <c r="X5" s="4" t="inlineStr">
+      <c r="Y5" s="4" t="inlineStr">
         <is>
           <t>Data verif.</t>
         </is>
       </c>
-      <c r="Y5" s="4" t="inlineStr">
+      <c r="Z5" s="4" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
@@ -1017,33 +1024,40 @@
       <c r="R6" s="9" t="n">
         <v>196222080</v>
       </c>
-      <c r="S6" s="10" t="n"/>
+      <c r="S6" s="10" t="n">
+        <v>0.515625</v>
+      </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
+          <t>calculado_automatico</t>
+        </is>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U6" s="6" t="inlineStr">
+      <c r="V6" s="6" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V6" s="6" t="inlineStr">
+      <c r="W6" s="6" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="W6" s="6" t="inlineStr">
+      <c r="X6" s="6" t="inlineStr">
         <is>
           <t>https://delman.com.br/maranhao/empreendimentos/proximos-lancamentos/edificio-the-view</t>
         </is>
       </c>
-      <c r="X6" s="6" t="inlineStr">
+      <c r="Y6" s="6" t="inlineStr">
         <is>
           <t>28/04/2026</t>
         </is>
       </c>
-      <c r="Y6" s="7" t="inlineStr">
+      <c r="Z6" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Studio a 3Q (1Q/2Q dominantes). PRÉ-LANÇAMENTO. Tabela atualizada 28/04/2026 (v3, versão 0000001 - 1.1). 13 pavtos tipo úteis (4º a 17º, exceto 10º — andar técnico/lazer). 93 aptos residenciais disponíveis + 1 loja (LOJA 21, 48,02m², R$890k). Tipologias 36,05–85,87 m² + cobertura 17º (5 aptos diferenciados 54-80m²). Estimativa ~49% vendido (assumindo ~182 unidades totais = 13 andares × 14 aptos). Ticket_min CAI para R$540k (apto 414, 36,45m²) — vs R$559k em 27/04 (apto que era min vendido OU apto 414 voltou ao mercado). Histórico tabelas: v1 24/04 (~110 disp.) → v2 27/04 (90 disp.) → v3 28/04 (93 disp. — leve recuperação, possível desistência de reserva). Parcelamento 100m + INCC/IGP-M+1%. Vista mar Calhau. VIZINHO ao Edifício Bossa (Mota Machado, mesma quadra 02 da Av. dos Holandeses).</t>
         </is>
@@ -1113,30 +1127,35 @@
       <c r="S7" s="16" t="n"/>
       <c r="T7" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U7" s="12" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="U7" s="12" t="inlineStr">
+      <c r="V7" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V7" s="12" t="inlineStr">
+      <c r="W7" s="12" t="inlineStr">
         <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W7" s="12" t="inlineStr">
+      <c r="X7" s="12" t="inlineStr">
         <is>
           <t>https://www.ergus.com.br</t>
         </is>
       </c>
-      <c r="X7" s="12" t="inlineStr">
+      <c r="Y7" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y7" s="13" t="inlineStr">
+      <c r="Z7" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Studio a 2Q. Complexo 10mil m² multi-produto (residencial + comercial + Open Mall). Book local + site oficial.</t>
         </is>
@@ -1200,30 +1219,35 @@
       <c r="S8" s="10" t="n"/>
       <c r="T8" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="U8" s="6" t="inlineStr">
+      <c r="V8" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
+      <c r="W8" s="6" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W8" s="6" t="inlineStr">
+      <c r="X8" s="6" t="inlineStr">
         <is>
           <t>https://construtoraluanova.com.br</t>
         </is>
       </c>
-      <c r="X8" s="6" t="inlineStr">
+      <c r="Y8" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y8" s="7" t="inlineStr">
+      <c r="Z8" s="7" t="inlineStr">
         <is>
           <t>Residência no Santo Amaro — região com oferta crescente de médio padrão.</t>
         </is>
@@ -1309,30 +1333,35 @@
       </c>
       <c r="T9" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U9" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U9" s="12" t="inlineStr">
+      <c r="V9" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V9" s="12" t="inlineStr">
+      <c r="W9" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="W9" s="12" t="inlineStr">
+      <c r="X9" s="12" t="inlineStr">
         <is>
           <t>https://motamachado.com.br</t>
         </is>
       </c>
-      <c r="X9" s="12" t="inlineStr">
+      <c r="Y9" s="12" t="inlineStr">
         <is>
           <t>28/04/2026</t>
         </is>
       </c>
-      <c r="Y9" s="13" t="inlineStr">
+      <c r="Z9" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 4 suítes (1 master c/ varanda, closet, banheiro duplo) + lavabo + varanda gourmet + qto/WC serviço. LANÇAMENTO 04/2026 — evento oficial 09/04/2026 (Frisson, MaHoje, Portal IN). 2 torres (Harmonia + Sintonia) × 15 pavtos tipo × 2 aptos/andar = 60 aptos. 6 elevadores. 3 tipologias: 191,02 / 192,64 / 196,04 m². 3 vagas (até 12º andar) ou 4 vagas (13º+ premium). Tabela 04/2026: 36 aptos disponíveis (24 vendidos = 40%). Tickets R$ 2,85-3,71M. R$/m² médio R$ 16.663 (faixa 14,9-19,2k — andares altos finais 01/02 tocam Luxo). Entrega 09/2030 (T-53). Memorial R 01, Matrícula 134.922 - 1º RI SL. **Projeto Arquitetônico: Nasser Hissa Arquitetos Associados** (parceiro recorrente em alto padrão). Lazer: brinquedoteca, salão festas, academia, pista funcional, quadra, lounge champanheira, piscina, pet wash, minimercado, estação carro elétrico. Mota Machado (CE) expandindo no NE, VGV 2025 R$350M. **VIZINHO ao The View (Delman, Lote 08 da mesma Quadra 02 — ambos na Av. dos Holandeses, Calhau)** — competição direta lado-a-lado, ambos lançados em 04/2026 mas com posicionamentos distintos: Bossa 4-suítes 191m² alto-padrão luxo vs The View Studio-3D 36-86m² médio-alto/alto.</t>
         </is>
@@ -1413,33 +1442,40 @@
       <c r="R10" s="9" t="n">
         <v>43086920.5</v>
       </c>
-      <c r="S10" s="10" t="n"/>
+      <c r="S10" s="10" t="n">
+        <v>0.1219512195121951</v>
+      </c>
       <c r="T10" s="6" t="inlineStr">
         <is>
+          <t>calculado_automatico</t>
+        </is>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U10" s="6" t="inlineStr">
+      <c r="V10" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V10" s="6" t="inlineStr">
+      <c r="W10" s="6" t="inlineStr">
         <is>
           <t>book</t>
         </is>
       </c>
-      <c r="W10" s="6" t="inlineStr">
+      <c r="X10" s="6" t="inlineStr">
         <is>
           <t>https://construtoracastelucci.com.br</t>
         </is>
       </c>
-      <c r="X10" s="6" t="inlineStr">
+      <c r="Y10" s="6" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y10" s="7" t="inlineStr">
+      <c r="Z10" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Casa 124,63 m² (terreno 164-204 m²). Tabela LANÇAMENTO 03/2026. Parceria Castelucci + Grupo Coimbra Alves. ~36-41 casas no Araçagi (numeração até casa 41, várias agrupadas: 02-17, 36-38, 39-40). Área construída UNIFORME 124,63 m². Terreno varia 164-204 m². Ticket à vista R$ 1.019.834 (casa 21) a R$ 1.081.967 (casa 41) — VARIAÇÃO POR TAMANHO DE TERRENO, não por área construída. Avaliação: R$ 915.000. Pagamento: 24m IPCA+0,49% / 36m IPCA+1,49% / Caixa. Lazer privativa não integrada ao preço. Paulo Castelucci (CEO) em entrevista à Mirante FM. Patrocínio Imob Summit 2026.</t>
         </is>
@@ -1525,30 +1561,35 @@
       </c>
       <c r="T11" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U11" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U11" s="12" t="inlineStr">
+      <c r="V11" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V11" s="12" t="inlineStr">
+      <c r="W11" s="12" t="inlineStr">
         <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W11" s="12" t="inlineStr">
+      <c r="X11" s="12" t="inlineStr">
         <is>
           <t>https://www.delman.com.br</t>
         </is>
       </c>
-      <c r="X11" s="12" t="inlineStr">
+      <c r="Y11" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y11" s="13" t="inlineStr">
+      <c r="Z11" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3 suítes. Tabela 04/2026 marcada 'pré-lançamento'. Fonte web confirma lançamento 2026. Duplex cobertura 123-143m².</t>
         </is>
@@ -1624,26 +1665,31 @@
       <c r="S12" s="10" t="n"/>
       <c r="T12" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U12" s="6" t="inlineStr">
+      <c r="V12" s="6" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr">
+      <c r="W12" s="6" t="inlineStr">
         <is>
           <t>interno</t>
         </is>
       </c>
-      <c r="W12" s="6" t="inlineStr"/>
-      <c r="X12" s="6" t="inlineStr">
+      <c r="X12" s="6" t="inlineStr"/>
+      <c r="Y12" s="6" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y12" s="7" t="inlineStr">
+      <c r="Z12" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Casa 3 dorm (1 suíte) + 2 vagas. Condomínio horizontal (sobrados). 1 ÚNICA tipologia: casa 100,35 m² construída (área usada para R$/m²). Terreno varia 136-146 m² conforme posição. ~38 casas. Lazer: campo society, piscina, deck, salão, gourmet, petplay, playground. Muitas unidades VENDIDAS. Entrega 01/2029. Ticket R$ 835-851k → R$/m² construção ~R$ 8.400. CORREÇÃO v5.2: Área máx era 145,78 (terreno) — corrigida para 100,35 (construída). Convenção PADRAO §1: Tipo=Horizontal usa área construída.</t>
         </is>
@@ -1729,20 +1775,25 @@
       </c>
       <c r="V13" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W13" s="12" t="inlineStr">
+        <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W13" s="12" t="inlineStr">
+      <c r="X13" s="12" t="inlineStr">
         <is>
           <t>https://www.instagram.com/mbengenharia.br/</t>
         </is>
       </c>
-      <c r="X13" s="12" t="inlineStr">
+      <c r="Y13" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y13" s="13" t="inlineStr">
+      <c r="Z13" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Casas duplex. 22 casas duplex 140m² — produto horizontal diferenciado. Pré-lançamento anunciado 2023, hoje em comercialização.</t>
         </is>
@@ -1826,30 +1877,35 @@
       <c r="S14" s="10" t="n"/>
       <c r="T14" s="6" t="inlineStr">
         <is>
+          <t>nao_determinavel</t>
+        </is>
+      </c>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U14" s="6" t="inlineStr">
+      <c r="V14" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V14" s="6" t="inlineStr">
+      <c r="W14" s="6" t="inlineStr">
         <is>
           <t>estimativa_T-36</t>
         </is>
       </c>
-      <c r="W14" s="6" t="inlineStr">
+      <c r="X14" s="6" t="inlineStr">
         <is>
           <t>https://www.niagara-imoveis.com.br</t>
         </is>
       </c>
-      <c r="X14" s="6" t="inlineStr">
+      <c r="Y14" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y14" s="7" t="inlineStr">
+      <c r="Z14" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2-4 suítes. Tabela JAN/26 é matriz por posição (não espelha estoque). Duplex cobertura 160m². Parcelamento 48m pós-assinatura.</t>
         </is>
@@ -1923,20 +1979,25 @@
       </c>
       <c r="V15" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W15" s="12" t="inlineStr">
+        <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W15" s="12" t="inlineStr">
+      <c r="X15" s="12" t="inlineStr">
         <is>
           <t>https://canopusconstrucoes.com.br</t>
         </is>
       </c>
-      <c r="X15" s="12" t="inlineStr">
+      <c r="Y15" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y15" s="13" t="inlineStr">
+      <c r="Z15" s="13" t="inlineStr">
         <is>
           <t>Série Village (estratégia de marca clara). Imirante 31/10/2025. Confirmar tipologia/ticket via site+IG.</t>
         </is>
@@ -2010,20 +2071,25 @@
       </c>
       <c r="V16" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W16" s="6" t="inlineStr">
+        <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W16" s="6" t="inlineStr">
+      <c r="X16" s="6" t="inlineStr">
         <is>
           <t>https://canopusconstrucoes.com.br</t>
         </is>
       </c>
-      <c r="X16" s="6" t="inlineStr">
+      <c r="Y16" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y16" s="7" t="inlineStr">
+      <c r="Z16" s="7" t="inlineStr">
         <is>
           <t>Canopus em movimento forte no Eldorado. Fonte: Imirante 31/10/2025.</t>
         </is>
@@ -2097,20 +2163,25 @@
       </c>
       <c r="V17" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W17" s="12" t="inlineStr">
+        <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W17" s="12" t="inlineStr">
+      <c r="X17" s="12" t="inlineStr">
         <is>
           <t>https://canopusconstrucoes.com.br</t>
         </is>
       </c>
-      <c r="X17" s="12" t="inlineStr">
+      <c r="Y17" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y17" s="13" t="inlineStr">
+      <c r="Z17" s="13" t="inlineStr">
         <is>
           <t>1 dos 3 novos lançamentos Canopus anunciados em 31/10/2025 (Imirante). SEM tabela ou book mapeado.</t>
         </is>
@@ -2174,30 +2245,35 @@
       <c r="S18" s="10" t="n"/>
       <c r="T18" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U18" s="6" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="U18" s="6" t="inlineStr">
+      <c r="V18" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V18" s="6" t="inlineStr">
+      <c r="W18" s="6" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W18" s="6" t="inlineStr">
+      <c r="X18" s="6" t="inlineStr">
         <is>
           <t>https://www.instagram.com/sacavalcantema/</t>
         </is>
       </c>
-      <c r="X18" s="6" t="inlineStr">
+      <c r="Y18" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y18" s="7" t="inlineStr">
+      <c r="Z18" s="7" t="inlineStr">
         <is>
           <t>Lançamento Sá Cavalcante out/2025. Estande 'Casa Sal' na Península. 'Os espaços conversam...' — narrativa de estilo de vida.</t>
         </is>
@@ -2283,30 +2359,35 @@
       </c>
       <c r="T19" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U19" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U19" s="12" t="inlineStr">
+      <c r="V19" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V19" s="12" t="inlineStr">
+      <c r="W19" s="12" t="inlineStr">
         <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W19" s="12" t="inlineStr">
+      <c r="X19" s="12" t="inlineStr">
         <is>
           <t>https://www.delman.com.br</t>
         </is>
       </c>
-      <c r="X19" s="12" t="inlineStr">
+      <c r="Y19" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y19" s="13" t="inlineStr">
+      <c r="Z19" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 4 suítes. Evento de apresentação oficial 2024. 5 de 30 à venda. ≈83% vendido. Piscina privativa na varanda.</t>
         </is>
@@ -2388,34 +2469,39 @@
         <v>141820500</v>
       </c>
       <c r="S20" s="10" t="n">
-        <v>0.17</v>
+        <v>0.833</v>
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U20" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U20" s="6" t="inlineStr">
+      <c r="V20" s="6" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V20" s="6" t="inlineStr">
+      <c r="W20" s="6" t="inlineStr">
         <is>
           <t>treinamento_corretor</t>
         </is>
       </c>
-      <c r="W20" s="6" t="inlineStr">
+      <c r="X20" s="6" t="inlineStr">
         <is>
           <t>https://www.ergus.com.br</t>
         </is>
       </c>
-      <c r="X20" s="6" t="inlineStr">
+      <c r="Y20" s="6" t="inlineStr">
         <is>
           <t>02/05/2026</t>
         </is>
       </c>
-      <c r="Y20" s="7" t="inlineStr">
+      <c r="Z20" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 4 suítes + 3 vagas. 2 torres × 14 pavtos tipo × 2 aptos/andar (Coluna 1 + Coluna 2) = 56 aptos no edifício. **TABELA 04/2026 EXTRAÍDA VIA VISÃO MULTIMODAL (v8.2 — 02/05/2026)** a partir do PDF imagem (pdftoppm + Claude visão). Tabela mostra 10 unidades disponíveis: Torre 1 col 1: aptos 202, 1101, 1201, 1202, 1301, 1501 (R$2.170k-2.557k); Torre 2 col 1: aptos 302, 1102, 1202 (R$2.192k-2.445k). Todas 148,55m² (4D suítes uniforme). R$/m² 14.610-17.212 (média ~R$15.500). Estimativa total ~60 unid. % Vendido estimado 83%. Memorial Reg. nº 02, Matrícula 130.345, 1º Cartório SL. Nota da tabela: obra entregue DEZ/26 mas unidades vendidas após ABRIL/26 serão entregues JUN/27 — sinal de tração tardia.</t>
         </is>
@@ -2489,20 +2575,25 @@
       </c>
       <c r="V21" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W21" s="12" t="inlineStr">
+        <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W21" s="12" t="inlineStr">
+      <c r="X21" s="12" t="inlineStr">
         <is>
           <t>https://www.bergengenharia.com.br</t>
         </is>
       </c>
-      <c r="X21" s="12" t="inlineStr">
+      <c r="Y21" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y21" s="13" t="inlineStr">
+      <c r="Z21" s="13" t="inlineStr">
         <is>
           <t>SPE Berg + Gonçalves requereu Licença de Instalação (Diário Oficial SL).</t>
         </is>
@@ -2586,30 +2677,35 @@
       <c r="S22" s="10" t="n"/>
       <c r="T22" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
           <t>book</t>
         </is>
       </c>
-      <c r="U22" s="6" t="inlineStr">
+      <c r="V22" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V22" s="6" t="inlineStr">
+      <c r="W22" s="6" t="inlineStr">
         <is>
           <t>book</t>
         </is>
       </c>
-      <c r="W22" s="6" t="inlineStr">
+      <c r="X22" s="6" t="inlineStr">
         <is>
           <t>https://construtoraluanova.com.br</t>
         </is>
       </c>
-      <c r="X22" s="6" t="inlineStr">
+      <c r="Y22" s="6" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y22" s="7" t="inlineStr">
+      <c r="Z22" s="7" t="inlineStr">
         <is>
           <t>LOTEAMENTO DE LUXO. Projeto Golden Green Beach (GGB) — bairro de luxo planejado, acesso pela Av. dos Holandeses. Lote 41: 453 m² R$ 2,65M (R$ 5.850/m² terreno). Lote 42: 682 m² R$ 4,40M (R$ 6.452/m² terreno). Em obra. Áreas comuns: piscina coberta aquecida, sauna a vapor, heliponto com acesso por escada e elevador, estacionamento 30 carros, área administrativa. Projeto arquitetônico das áreas comuns: Marcelo Franco. Urbanismo: SA Urbanismo. Referências de luxo (book): Porto Frade RJ, Fazenda Boa Vista SP, Quinta da Baroneza SP. Bairro a confirmar (Calhau ou São Marcos pela posição na Av. Holandeses). ATENÇÃO: R$/m² em loteamento é TERRENO, não construído — não compara diretamente com aptos.</t>
         </is>
@@ -2695,30 +2791,35 @@
       </c>
       <c r="T23" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U23" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U23" s="12" t="inlineStr">
+      <c r="V23" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V23" s="12" t="inlineStr">
+      <c r="W23" s="12" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W23" s="12" t="inlineStr">
+      <c r="X23" s="12" t="inlineStr">
         <is>
           <t>https://monteplanengenharia.com.br/empreendimentos/renaissance-conceito/</t>
         </is>
       </c>
-      <c r="X23" s="12" t="inlineStr">
+      <c r="Y23" s="12" t="inlineStr">
         <is>
           <t>29/04/2026</t>
         </is>
       </c>
-      <c r="Y23" s="13" t="inlineStr">
+      <c r="Z23" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2 torres × 15 pav. tipo. **Torre Leonardo da Vinci** 45 unid (3 aptos/andar): 110m², 3 SUÍTES + lavabo, 2 ou 3 vagas (1º-5º andar 2 vagas / 6º-15º 3 vagas). **Torre Botticelli** 60 unid (4 aptos/andar): 82m², 3 quartos (2 suítes, sendo 1 reversível), 2 vagas. Total 105 unidades. Tabela 04/2026 lista 22 unidades LIVRES (15 Botticelli + 7 Leonardo) — assumindo que tabela só lista LIVRES, estimativa 79% vendido (margem: pode haver reservadas/contratadas não mostradas). Tickets R$ 1.038k (BO 101, menor) a R$ 1.565k (LE 1401, maior). Conclusão obra AGO/2027. Construtora Monteplan. Versão tabela 1.04.</t>
         </is>
@@ -2792,20 +2893,25 @@
       </c>
       <c r="V24" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W24" s="6" t="inlineStr">
+      <c r="X24" s="6" t="inlineStr">
         <is>
           <t>https://trevisoengenharia.com.br</t>
         </is>
       </c>
-      <c r="X24" s="6" t="inlineStr">
+      <c r="Y24" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y24" s="7" t="inlineStr">
+      <c r="Z24" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Terrenos em condomínio. Condomínio de terrenos (loteamento fechado). Divulgação ativa abr/2026. Sem tabela pública mapeada.</t>
         </is>
@@ -2891,30 +2997,35 @@
       </c>
       <c r="T25" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U25" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U25" s="12" t="inlineStr">
+      <c r="V25" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V25" s="12" t="inlineStr">
+      <c r="W25" s="12" t="inlineStr">
         <is>
           <t>estimativa_T-36</t>
         </is>
       </c>
-      <c r="W25" s="12" t="inlineStr">
+      <c r="X25" s="12" t="inlineStr">
         <is>
           <t>https://www.delman.com.br</t>
         </is>
       </c>
-      <c r="X25" s="12" t="inlineStr">
+      <c r="Y25" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y25" s="13" t="inlineStr">
+      <c r="Z25" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Studio / 1Q. 33 de 125 aptos à venda. ≈74% vendido em ~18 meses. Forte velocidade em compactos.</t>
         </is>
@@ -2995,29 +3106,36 @@
       <c r="R26" s="9" t="n">
         <v>19750000</v>
       </c>
-      <c r="S26" s="10" t="n"/>
+      <c r="S26" s="10" t="n">
+        <v>0.84</v>
+      </c>
       <c r="T26" s="6" t="inlineStr">
         <is>
+          <t>calculado_automatico</t>
+        </is>
+      </c>
+      <c r="U26" s="6" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U26" s="6" t="inlineStr">
+      <c r="V26" s="6" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V26" s="6" t="inlineStr">
+      <c r="W26" s="6" t="inlineStr">
         <is>
           <t>memorial</t>
         </is>
       </c>
-      <c r="W26" s="6" t="inlineStr"/>
-      <c r="X26" s="6" t="inlineStr">
+      <c r="X26" s="6" t="inlineStr"/>
+      <c r="Y26" s="6" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y26" s="7" t="inlineStr">
+      <c r="Z26" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Studios e 1-2 dorm (compactos premium). Parceria Hiali + Silveira Inc. Compactos premium: 49,74 / 58,91 / 62,62 m². 5 pavimentos tipo × 5 aptos/andar = ~25 unidades. Entrega DEZ/2027. Ticket R$ 710-870k. R$/m² méd R$ 13.810. Memorial R.09/25.101 registrado 17/04/2025 no 1º RI São Luís. Foco em mercado jovem / investidor. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -3103,30 +3221,35 @@
       </c>
       <c r="T27" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U27" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U27" s="12" t="inlineStr">
+      <c r="V27" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V27" s="12" t="inlineStr">
+      <c r="W27" s="12" t="inlineStr">
         <is>
           <t>memorial</t>
         </is>
       </c>
-      <c r="W27" s="12" t="inlineStr">
+      <c r="X27" s="12" t="inlineStr">
         <is>
           <t>https://www.instagram.com/alfaengenhariama/</t>
         </is>
       </c>
-      <c r="X27" s="12" t="inlineStr">
+      <c r="Y27" s="12" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y27" s="13" t="inlineStr">
+      <c r="Z27" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2 suítes + 2 semi-suítes OU 3 suítes, varanda, lavabo, 3 vagas, depósito. Torre NORTE do Giardino. 15 pav × 3 un = 45 unidades. 3 tipologias: 127,30 / 128,37 / 110,77 m². Tabela MAR/2026: 6 unidades disponíveis (1001/701/201/101 da coluna 127m², 102 da coluna 128m², 1403 da coluna 110m²) = ~13% estoque, 87% VENDIDO → Últimas unidades. Entrega DEZ/29. Memorial R.06/56.931 - 1º RI SL. Endereço Alfa: Rua Peixe Pedra, Qd 12 lote 04, Calhau.</t>
         </is>
@@ -3212,30 +3335,35 @@
       </c>
       <c r="T28" s="6" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U28" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U28" s="6" t="inlineStr">
+      <c r="V28" s="6" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V28" s="6" t="inlineStr">
+      <c r="W28" s="6" t="inlineStr">
         <is>
           <t>memorial</t>
         </is>
       </c>
-      <c r="W28" s="6" t="inlineStr">
+      <c r="X28" s="6" t="inlineStr">
         <is>
           <t>https://www.instagram.com/alfaengenhariama/</t>
         </is>
       </c>
-      <c r="X28" s="6" t="inlineStr">
+      <c r="Y28" s="6" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y28" s="7" t="inlineStr">
+      <c r="Z28" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3 suítes, varanda, lavabo, 2 vagas, depósito. Torre SUL do Giardino. 15 pav × 4 un = 60 unidades. 4 tipologias: 99,08 / 101,31 / 93,18 / 93,62 m². Tabela MAR/2026: 5 unidades disponíveis (701/101 col 99m², 1502/1402 col 101m², 104 col 93m²) = ~8% estoque, 92% VENDIDO → Últimas unidades. CORREÇÃO v5.1: dorms = 3 suítes (descrição da tabela MAR/26), antes constava '2 suítes/1 suíte' incorretamente. 2 vagas + 1 depósito. Mais acessível que Torre Fiore. Entrega DEZ/29. Memorial R.06/56.931 - 1º RI SL.</t>
         </is>
@@ -3317,34 +3445,39 @@
         <v>243300000</v>
       </c>
       <c r="S29" s="16" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="T29" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U29" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U29" s="12" t="inlineStr">
+      <c r="V29" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V29" s="12" t="inlineStr">
+      <c r="W29" s="12" t="inlineStr">
         <is>
           <t>informado</t>
         </is>
       </c>
-      <c r="W29" s="12" t="inlineStr">
+      <c r="X29" s="12" t="inlineStr">
         <is>
           <t>https://www.treviso.com.br</t>
         </is>
       </c>
-      <c r="X29" s="12" t="inlineStr">
+      <c r="Y29" s="12" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y29" s="13" t="inlineStr">
+      <c r="Z29" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Aptos 130 m² — Leste/Sul/Norte. Lançamento 02/2025 informado pelo Rafael (fonte externa confiável). Tabela de 02/2026 arquivada confirma vendas ativas naquela data, mas não é data de lançamento — aguarda book ou memorial para data confiável. Torre Norte: 37 unid, área 130 m², ticket R$ 1,82-2,24M (méd R$ 2,02M). R$/m² méd R$ 15.524. VGV listado R$ 74,8M. Entrega 12/2029. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -3425,33 +3558,40 @@
       <c r="R30" s="9" t="n">
         <v>85890000</v>
       </c>
-      <c r="S30" s="10" t="n"/>
+      <c r="S30" s="10" t="n">
+        <v>0.5666666666666667</v>
+      </c>
       <c r="T30" s="6" t="inlineStr">
         <is>
+          <t>calculado_automatico</t>
+        </is>
+      </c>
+      <c r="U30" s="6" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U30" s="6" t="inlineStr">
+      <c r="V30" s="6" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V30" s="6" t="inlineStr">
+      <c r="W30" s="6" t="inlineStr">
         <is>
           <t>informado</t>
         </is>
       </c>
-      <c r="W30" s="6" t="inlineStr">
+      <c r="X30" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="X30" s="6" t="inlineStr">
+      <c r="Y30" s="6" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y30" s="7" t="inlineStr">
+      <c r="Z30" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 87,98 e 90,10 m² (Norte/Sul). Lançamento 02/2025 informado pelo Rafael. 26 unid listadas, área 87,98/90,10 m². Ticket R$ 1,28-1,59M (méd R$ 1,40M). R$/m² pond R$ 15.600 (faixa R$ 14,2-17,6k). VGV listado R$ 36,3M. Entrega 12/2029. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -3532,33 +3672,40 @@
       <c r="R31" s="15" t="n">
         <v>103245615</v>
       </c>
-      <c r="S31" s="16" t="n"/>
+      <c r="S31" s="16" t="n">
+        <v>0.9333333333333333</v>
+      </c>
       <c r="T31" s="12" t="inlineStr">
         <is>
+          <t>calculado_automatico</t>
+        </is>
+      </c>
+      <c r="U31" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U31" s="12" t="inlineStr">
+      <c r="V31" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V31" s="12" t="inlineStr">
+      <c r="W31" s="12" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W31" s="12" t="inlineStr">
+      <c r="X31" s="12" t="inlineStr">
         <is>
           <t>https://www.motamachado.com.br</t>
         </is>
       </c>
-      <c r="X31" s="12" t="inlineStr">
+      <c r="Y31" s="12" t="inlineStr">
         <is>
           <t>29/04/2026</t>
         </is>
       </c>
-      <c r="Y31" s="13" t="inlineStr">
+      <c r="Z31" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2 torres (Litorânea + Lagoa). **Planta 1** (67,48-68,75m²) — 2D: 1 quarto + 1 suíte de casal, varanda gourmet, 1-2 vagas. **Planta 2** (102,25-104,05m²) — 3D: 2 suítes + suíte de casal, varanda gourmet, 1 vaga. Tabela 04/2026 PRÉ-LANÇAMENTO mostra preços por andar (plano 60% mensal): R$977k (Lagoa 301-303) a R$1.317k (Litorânea 1701-1703). Plano 100% mensais (com juros embutidos) chega a R$1,87M. Áreas extraídas do BOOK — tabela em si não traz m². Projeto IDEA (Fabián Salles), paisagismo Beth Miyazaki, interiores Sobre Arquitetura. Entrega 28/02/2029 (T-49 desde lançamento 01/2025). % Vendido não calculado: tabela é PRÉ-LANÇAMENTO, sem total de unidades visível. Mota Machado (Fortaleza/CE) — Empresa expandindo no Nordeste.</t>
         </is>
@@ -3644,30 +3791,35 @@
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U32" s="6" t="inlineStr">
+      <c r="V32" s="6" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V32" s="6" t="inlineStr">
+      <c r="W32" s="6" t="inlineStr">
         <is>
           <t>estimativa_T-36</t>
         </is>
       </c>
-      <c r="W32" s="6" t="inlineStr">
+      <c r="X32" s="6" t="inlineStr">
         <is>
           <t>https://www.delman.com.br</t>
         </is>
       </c>
-      <c r="X32" s="6" t="inlineStr">
+      <c r="Y32" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y32" s="7" t="inlineStr">
+      <c r="Z32" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 4 suítes. Prédio pequeno (12 aptos). 1 à venda. ≈92% vendido.</t>
         </is>
@@ -3747,30 +3899,35 @@
       <c r="S33" s="16" t="n"/>
       <c r="T33" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U33" s="12" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U33" s="12" t="inlineStr">
+      <c r="V33" s="12" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V33" s="12" t="inlineStr">
+      <c r="W33" s="12" t="inlineStr">
         <is>
           <t>book</t>
         </is>
       </c>
-      <c r="W33" s="12" t="inlineStr">
+      <c r="X33" s="12" t="inlineStr">
         <is>
           <t>https://motamachado.com.br</t>
         </is>
       </c>
-      <c r="X33" s="12" t="inlineStr">
+      <c r="Y33" s="12" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y33" s="13" t="inlineStr">
+      <c r="Z33" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 4 suítes, 3 vagas. Torre A 'Tirreno' da Mota Machado Collection. Imóvel PRONTO. 215 m², 4 suítes, 3 vagas. Apts 102, 201, 202 listados. Ticket R$ 3,02-3,12M. R$/m² méd R$ 14.293. Av. dos Holandeses / São Marcos. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -3851,33 +4008,40 @@
       <c r="R34" s="9" t="n">
         <v>66780000</v>
       </c>
-      <c r="S34" s="10" t="n"/>
+      <c r="S34" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="T34" s="6" t="inlineStr">
         <is>
+          <t>tabela_local_completa_zero</t>
+        </is>
+      </c>
+      <c r="U34" s="6" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U34" s="6" t="inlineStr">
+      <c r="V34" s="6" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V34" s="6" t="inlineStr">
+      <c r="W34" s="6" t="inlineStr">
         <is>
           <t>book</t>
         </is>
       </c>
-      <c r="W34" s="6" t="inlineStr">
+      <c r="X34" s="6" t="inlineStr">
         <is>
           <t>https://motamachado.com.br</t>
         </is>
       </c>
-      <c r="X34" s="6" t="inlineStr">
+      <c r="Y34" s="6" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y34" s="7" t="inlineStr">
+      <c r="Z34" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3 suítes (1 master). 3 tipologias (125 / 146,82 / 156,94 m²). 2 torres x 15 pav. Tab ABR/26: 15 unid, VGV R$ 32,3M. Ticket R$ 1,73–2,72M (méd R$ 2,15M). R$/m² pond R$ 15.162 (faixa R$ 13,9k–17,3k). Rua dos Bicudos, Renascença. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -3951,20 +4115,25 @@
       </c>
       <c r="V35" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W35" s="12" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W35" s="12" t="inlineStr">
+      <c r="X35" s="12" t="inlineStr">
         <is>
           <t>https://www.alfaengenharia.com.br</t>
         </is>
       </c>
-      <c r="X35" s="12" t="inlineStr">
+      <c r="Y35" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y35" s="13" t="inlineStr">
+      <c r="Z35" s="13" t="inlineStr">
         <is>
           <t>Tipologia a confirmar em book/site/Instagram. Tecnologia Housi (gestão de locação) NÃO determina tipologia — descrição anterior corrigida. Sem tabela comercial pública.</t>
         </is>
@@ -4038,20 +4207,25 @@
       </c>
       <c r="V36" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W36" s="6" t="inlineStr">
+        <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W36" s="6" t="inlineStr">
+      <c r="X36" s="6" t="inlineStr">
         <is>
           <t>https://www.alfaengenharia.com.br</t>
         </is>
       </c>
-      <c r="X36" s="6" t="inlineStr">
+      <c r="Y36" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y36" s="7" t="inlineStr">
+      <c r="Z36" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 4 suítes. 13 opções de lazer, elevador privativo. Book local (375MB) + site oficial. Sem ticket público.</t>
         </is>
@@ -4121,30 +4295,35 @@
       <c r="S37" s="16" t="n"/>
       <c r="T37" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U37" s="12" t="inlineStr">
+        <is>
           <t>agregador</t>
         </is>
       </c>
-      <c r="U37" s="12" t="inlineStr">
+      <c r="V37" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V37" s="12" t="inlineStr">
+      <c r="W37" s="12" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W37" s="12" t="inlineStr">
+      <c r="X37" s="12" t="inlineStr">
         <is>
           <t>https://construtoracastelucci.com.br</t>
         </is>
       </c>
-      <c r="X37" s="12" t="inlineStr">
+      <c r="Y37" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y37" s="13" t="inlineStr">
+      <c r="Z37" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2Q. Compactos 49-52m², 2Q. Público Cohatrac/médio. Instagram @construtoracastelucci anunciou como lançamento; preço não divulgado.</t>
         </is>
@@ -4220,26 +4399,31 @@
       <c r="S38" s="10" t="n"/>
       <c r="T38" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U38" s="6" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U38" s="6" t="inlineStr">
+      <c r="V38" s="6" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V38" s="6" t="inlineStr">
+      <c r="W38" s="6" t="inlineStr">
         <is>
           <t>interno</t>
         </is>
       </c>
-      <c r="W38" s="6" t="inlineStr"/>
-      <c r="X38" s="6" t="inlineStr">
+      <c r="X38" s="6" t="inlineStr"/>
+      <c r="Y38" s="6" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y38" s="7" t="inlineStr">
+      <c r="Z38" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Casa 4+ dorm, alto padrão. Condomínio horizontal alto padrão. 1 ÚNICA tipologia: casa 154,64 m² construída. Terreno varia 170-181 m² conforme posição. Maioria das unidades VENDIDAS (14+ marcadas VENDIDA na tabela ABR/2026). Entrega 06/2027. Ticket ~R$ 1,4M → R$/m² construção ~R$ 9.150. CORREÇÃO v5.2: Área máx era 180,98 (terreno) — corrigida para 154,64 (construída). Convenção PADRAO §1: Tipo=Horizontal usa área construída.</t>
         </is>
@@ -4303,30 +4487,35 @@
       <c r="S39" s="16" t="n"/>
       <c r="T39" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U39" s="12" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="U39" s="12" t="inlineStr">
+      <c r="V39" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V39" s="12" t="inlineStr">
+      <c r="W39" s="12" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W39" s="12" t="inlineStr">
+      <c r="X39" s="12" t="inlineStr">
         <is>
           <t>https://franere.com.br</t>
         </is>
       </c>
-      <c r="X39" s="12" t="inlineStr">
+      <c r="Y39" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y39" s="13" t="inlineStr">
+      <c r="Z39" s="13" t="inlineStr">
         <is>
           <t>Franere ('Maior construtora do Maranhão', 40 anos). Série 'Gran Park' tem múltiplos módulos. IG @franereoficial_.</t>
         </is>
@@ -4390,30 +4579,35 @@
       <c r="S40" s="10" t="n"/>
       <c r="T40" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U40" s="6" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="U40" s="6" t="inlineStr">
+      <c r="V40" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V40" s="6" t="inlineStr">
+      <c r="W40" s="6" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W40" s="6" t="inlineStr">
+      <c r="X40" s="6" t="inlineStr">
         <is>
           <t>https://construtoraluanova.com.br</t>
         </is>
       </c>
-      <c r="X40" s="6" t="inlineStr">
+      <c r="Y40" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y40" s="7" t="inlineStr">
+      <c r="Z40" s="7" t="inlineStr">
         <is>
           <t>Construtora Lua Nova desde 1985. IG @construtoraluanova. Detalhes tipologia/ticket a coletar via book.</t>
         </is>
@@ -4489,30 +4683,35 @@
       <c r="S41" s="16" t="n"/>
       <c r="T41" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U41" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U41" s="12" t="inlineStr">
+      <c r="V41" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V41" s="12" t="inlineStr">
+      <c r="W41" s="12" t="inlineStr">
         <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W41" s="12" t="inlineStr">
+      <c r="X41" s="12" t="inlineStr">
         <is>
           <t>https://www.bergengenharia.com.br</t>
         </is>
       </c>
-      <c r="X41" s="12" t="inlineStr">
+      <c r="Y41" s="12" t="inlineStr">
         <is>
           <t>27/04/2026</t>
         </is>
       </c>
-      <c r="Y41" s="13" t="inlineStr">
+      <c r="Z41" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: Aptos 135 m², 2-3 vagas. Tabela ABR/2026 (Berg Engenharia). 4 tipologias (1-4) com áreas similares 135,32 / 135,83 m². Lançamento 04/2024 estimado pela pasta. Conclusão: 30/04/2027 (T-36 perfeito). Tipo 3 (135,32m²): apto 103 disponível R$ 1.932.400. Tipo 4 (135,83m²): apto 104 disponível R$ 1.944.500, demais (204-1004) VENDIDOS = 9 vendidos no Tipo 4 → estoque concentrado em 1 unidade visível. Apto 704 tem 3 vagas (diferencial). Correção INCC. Histórico Berg: Montparnasse, Golden Tower, Peninsula Mall, Monte Olimpo, Monte Fuji.</t>
         </is>
@@ -4593,33 +4792,40 @@
       <c r="R42" s="9" t="n">
         <v>16347500</v>
       </c>
-      <c r="S42" s="10" t="n"/>
+      <c r="S42" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="T42" s="6" t="inlineStr">
         <is>
+          <t>calculado_automatico</t>
+        </is>
+      </c>
+      <c r="U42" s="6" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U42" s="6" t="inlineStr">
+      <c r="V42" s="6" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V42" s="6" t="inlineStr">
+      <c r="W42" s="6" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="W42" s="6" t="inlineStr">
+      <c r="X42" s="6" t="inlineStr">
         <is>
           <t>https://trevisoengenharia.com.br</t>
         </is>
       </c>
-      <c r="X42" s="6" t="inlineStr">
+      <c r="Y42" s="6" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y42" s="7" t="inlineStr">
+      <c r="Z42" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2-3Q (1 ou 2 vagas). IMÓVEL PRONTO. 26+ unid na tab ABR/26 (VGV R$ 15,8M). Tipos: 57,93 m² (1 vaga) e 67,15 m² (2 vagas). Ticket R$ 495k–762k (méd R$ 607k). R$/m² pond R$ 10.042. Estoque amplo. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -4691,30 +4897,35 @@
       </c>
       <c r="T43" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U43" s="12" t="inlineStr">
+        <is>
           <t>agregador</t>
         </is>
       </c>
-      <c r="U43" s="12" t="inlineStr">
+      <c r="V43" s="12" t="inlineStr">
         <is>
           <t>agregador</t>
         </is>
       </c>
-      <c r="V43" s="12" t="inlineStr">
+      <c r="W43" s="12" t="inlineStr">
         <is>
           <t>interno</t>
         </is>
       </c>
-      <c r="W43" s="12" t="inlineStr">
+      <c r="X43" s="12" t="inlineStr">
         <is>
           <t>https://www.imeu.com.br/empreendimento/dom-ricardo-apartamentos-sao-luis-2-a-3-quartos-71-a-85-m/19044585-MIM</t>
         </is>
       </c>
-      <c r="X43" s="12" t="inlineStr">
+      <c r="Y43" s="12" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y43" s="13" t="inlineStr">
+      <c r="Z43" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2-3Q. DOM Incorporação com MB Engenharia como sócia (empreendimento conjunto). Lançamento 12/2023 confirmado internamente. Próximo à Praça da Lagoa (Foguete). 'Sucesso de vendas, 6 unidades disponíveis' (IG jan/2025). Estoque estimado ≤6%. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -4788,20 +4999,25 @@
       </c>
       <c r="V44" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W44" s="6" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W44" s="6" t="inlineStr">
+      <c r="X44" s="6" t="inlineStr">
         <is>
           <t>https://www.alfaengenharia.com.br</t>
         </is>
       </c>
-      <c r="X44" s="6" t="inlineStr">
+      <c r="Y44" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y44" s="7" t="inlineStr">
+      <c r="Z44" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3 suítes. 1º Housi do MA. Book local + site Alfa. Sem tabela comercial.</t>
         </is>
@@ -4887,30 +5103,35 @@
       </c>
       <c r="T45" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U45" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U45" s="12" t="inlineStr">
+      <c r="V45" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V45" s="12" t="inlineStr">
+      <c r="W45" s="12" t="inlineStr">
         <is>
           <t>imprensa</t>
         </is>
       </c>
-      <c r="W45" s="12" t="inlineStr">
+      <c r="X45" s="12" t="inlineStr">
         <is>
           <t>https://www.delman.com.br</t>
         </is>
       </c>
-      <c r="X45" s="12" t="inlineStr">
+      <c r="Y45" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y45" s="13" t="inlineStr">
+      <c r="Z45" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3 suítes. Tabela 04/2026: 1 apto (901) de 30. ≈97% vendido. Lançamento confirmado 2023 pela imprensa.</t>
         </is>
@@ -4986,30 +5207,35 @@
       <c r="S46" s="10" t="n"/>
       <c r="T46" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U46" s="6" t="inlineStr">
+        <is>
           <t>agregador</t>
         </is>
       </c>
-      <c r="U46" s="6" t="inlineStr">
+      <c r="V46" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V46" s="6" t="inlineStr">
+      <c r="W46" s="6" t="inlineStr">
         <is>
           <t>interno</t>
         </is>
       </c>
-      <c r="W46" s="6" t="inlineStr">
+      <c r="X46" s="6" t="inlineStr">
         <is>
           <t>https://www.imovelnacidade.com/destaque/mb-construtora/</t>
         </is>
       </c>
-      <c r="X46" s="6" t="inlineStr">
+      <c r="Y46" s="6" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y46" s="7" t="inlineStr">
+      <c r="Z46" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3Q casas duplex. DOM Incorporação com MB Engenharia como sócia (empreendimento conjunto). Lançamento 06/2023 confirmado internamente. Casa duplex 3Q, 136m², R$906.870. Produto horizontal Eldorado/Turú. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -5091,30 +5317,35 @@
       </c>
       <c r="T47" s="12" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U47" s="12" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U47" s="12" t="inlineStr">
+      <c r="V47" s="12" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V47" s="12" t="inlineStr">
+      <c r="W47" s="12" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W47" s="12" t="inlineStr">
+      <c r="X47" s="12" t="inlineStr">
         <is>
           <t>https://monteplanengenharia.com.br/empreendimentos/edificio-sanpaolo/</t>
         </is>
       </c>
-      <c r="X47" s="12" t="inlineStr">
+      <c r="Y47" s="12" t="inlineStr">
         <is>
           <t>29/04/2026</t>
         </is>
       </c>
-      <c r="Y47" s="13" t="inlineStr">
+      <c r="Z47" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2 plantas. **Colunas 1,2,7,8** com 59m² — 3 quartos (1 suíte), 2 vagas. **Colunas 3,4,5,6** com 54m² — 2 quartos (2 suítes, sendo 1 reversível), 1 vaga. Tabela 04/2026 lista APENAS 1 unidade LIVRE (apto 204-205, R$ 610.000 — par de unidades unidas, situação L-L). Estimativa ≥98% vendido. Confirma 'todas as unidades vendidas' (Facebook out/2025) — restou só 1 unid. dupla. Endereço completo: Rua Boa Esperança, 125, Cohama (ao lado da Igreja Batista). Conclusão obra DEZ/2025.</t>
         </is>
@@ -5200,30 +5431,35 @@
       </c>
       <c r="T48" s="6" t="inlineStr">
         <is>
+          <t>informado_manualmente</t>
+        </is>
+      </c>
+      <c r="U48" s="6" t="inlineStr">
+        <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="U48" s="6" t="inlineStr">
+      <c r="V48" s="6" t="inlineStr">
         <is>
           <t>tabela_local</t>
         </is>
       </c>
-      <c r="V48" s="6" t="inlineStr">
+      <c r="W48" s="6" t="inlineStr">
         <is>
           <t>estimativa_T-36</t>
         </is>
       </c>
-      <c r="W48" s="6" t="inlineStr">
+      <c r="X48" s="6" t="inlineStr">
         <is>
           <t>https://www.delman.com.br</t>
         </is>
       </c>
-      <c r="X48" s="6" t="inlineStr">
+      <c r="Y48" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y48" s="7" t="inlineStr">
+      <c r="Z48" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 3 suítes. Entrega iminente. 1 apto (601) de 30 à venda. ≈97% vendido.</t>
         </is>
@@ -5299,30 +5535,35 @@
       <c r="S49" s="16" t="n"/>
       <c r="T49" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U49" s="12" t="inlineStr">
+        <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="U49" s="12" t="inlineStr">
+      <c r="V49" s="12" t="inlineStr">
         <is>
           <t>tabela</t>
         </is>
       </c>
-      <c r="V49" s="12" t="inlineStr">
+      <c r="W49" s="12" t="inlineStr">
         <is>
           <t>memorial</t>
         </is>
       </c>
-      <c r="W49" s="12" t="inlineStr">
+      <c r="X49" s="12" t="inlineStr">
         <is>
           <t>https://monteplanengenharia.com.br</t>
         </is>
       </c>
-      <c r="X49" s="12" t="inlineStr">
+      <c r="Y49" s="12" t="inlineStr">
         <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="Y49" s="13" t="inlineStr">
+      <c r="Z49" s="13" t="inlineStr">
         <is>
           <t>OBRA CONCLUÍDA (Monteplan, Cohab Anil IV). 32 unid listadas, todas ~R$ 324.142 (área 53,94 m²). R$/m² uniforme R$ 6.009. Padrão popular. SFH 60%. VGV residual listado R$ 10,4M. [reconstituído da v4.16 em 25/04/2026]</t>
         </is>
@@ -5408,20 +5649,25 @@
       </c>
       <c r="V50" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W50" s="6" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W50" s="6" t="inlineStr">
+      <c r="X50" s="6" t="inlineStr">
         <is>
           <t>https://www.sacavalcante.com.br</t>
         </is>
       </c>
-      <c r="X50" s="6" t="inlineStr">
+      <c r="Y50" s="6" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y50" s="7" t="inlineStr">
+      <c r="Z50" s="7" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2-3 quartos. 120 aptos (60 2Q + 60 3Q), 12/andar, 15 pavs. Pronto p/ morar. Ao lado do Shopping da Ilha.</t>
         </is>
@@ -5485,30 +5731,35 @@
       <c r="S51" s="16" t="n"/>
       <c r="T51" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U51" s="12" t="inlineStr">
+        <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="U51" s="12" t="inlineStr">
+      <c r="V51" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V51" s="12" t="inlineStr">
+      <c r="W51" s="12" t="inlineStr">
         <is>
           <t>site_oficial</t>
         </is>
       </c>
-      <c r="W51" s="12" t="inlineStr">
+      <c r="X51" s="12" t="inlineStr">
         <is>
           <t>https://construtoracastelucci.com.br</t>
         </is>
       </c>
-      <c r="X51" s="12" t="inlineStr">
+      <c r="Y51" s="12" t="inlineStr">
         <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="Y51" s="13" t="inlineStr">
+      <c r="Z51" s="13" t="inlineStr">
         <is>
           <t>Tipologia detalhada: 2-3Q. Apartamentos 2-3Q Araçagy. Site oficial Castelucci.</t>
         </is>
@@ -5529,12 +5780,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:Y51"/>
+  <autoFilter ref="A5:Z51"/>
   <mergeCells count="4">
-    <mergeCell ref="A52:Y52"/>
-    <mergeCell ref="D2:Y2"/>
-    <mergeCell ref="A53:Y53"/>
-    <mergeCell ref="D3:Y3"/>
+    <mergeCell ref="D3:Z3"/>
+    <mergeCell ref="D2:Z2"/>
+    <mergeCell ref="A52:Z52"/>
+    <mergeCell ref="A53:Z53"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>